<commit_message>
Set real player beam interval to half a second and preserve base throughput
</commit_message>
<xml_diff>
--- a/space-battleship/config_excel/equipment.xlsx
+++ b/space-battleship/config_excel/equipment.xlsx
@@ -1578,13 +1578,13 @@
         <v>1</v>
       </c>
       <c r="E12" s="0" t="n">
-        <v>35</v>
+        <v>62.5</v>
       </c>
       <c r="F12" s="0" t="n">
         <v>0.2</v>
       </c>
       <c r="G12" s="0" t="n">
-        <v>0.28</v>
+        <v>0.5</v>
       </c>
       <c r="I12" s="0" t="n">
         <v>1</v>

</xml_diff>

<commit_message>
Align missile base timing and mark dynamic interval estimates
</commit_message>
<xml_diff>
--- a/space-battleship/config_excel/equipment.xlsx
+++ b/space-battleship/config_excel/equipment.xlsx
@@ -1413,13 +1413,13 @@
         <v>2</v>
       </c>
       <c r="E7" s="0" t="n">
-        <v>200</v>
+        <v>208.5</v>
       </c>
       <c r="F7" s="0" t="n">
         <v>0.2</v>
       </c>
       <c r="G7" s="0" t="n">
-        <v>2.4</v>
+        <v>2.5</v>
       </c>
       <c r="I7" s="0" t="n">
         <v>1</v>

</xml_diff>

<commit_message>
Prepare integrated readability candidate and gated fresh-playtest workflow
</commit_message>
<xml_diff>
--- a/space-battleship/config_excel/equipment.xlsx
+++ b/space-battleship/config_excel/equipment.xlsx
@@ -1413,13 +1413,13 @@
         <v>2</v>
       </c>
       <c r="E7" s="0" t="n">
-        <v>200</v>
+        <v>208.5</v>
       </c>
       <c r="F7" s="0" t="n">
         <v>0.2</v>
       </c>
       <c r="G7" s="0" t="n">
-        <v>2.4</v>
+        <v>2.5</v>
       </c>
       <c r="I7" s="0" t="n">
         <v>1</v>

</xml_diff>

<commit_message>
balance: author opening 18 encounters and combat roles
</commit_message>
<xml_diff>
--- a/space-battleship/config_excel/equipment.xlsx
+++ b/space-battleship/config_excel/equipment.xlsx
@@ -1,12 +1,12 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr codeName="ThisWorkbook"/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" windowWidth="29868" windowHeight="13380" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="equipment" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="equipment" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
@@ -1374,13 +1374,13 @@
         <v>1</v>
       </c>
       <c r="E6" s="0" t="n">
-        <v>100</v>
+        <v>300</v>
       </c>
       <c r="F6" s="0" t="n">
         <v>0.2</v>
       </c>
       <c r="G6" s="0" t="n">
-        <v>0.5</v>
+        <v>1.5</v>
       </c>
       <c r="I6" s="0" t="n">
         <v>1</v>
@@ -1392,7 +1392,7 @@
         <v>0.2</v>
       </c>
       <c r="O6" s="0" t="n">
-        <v>30</v>
+        <v>10000</v>
       </c>
     </row>
     <row r="7">

</xml_diff>

<commit_message>
Set four weapon roles with safe precision limits
</commit_message>
<xml_diff>
--- a/space-battleship/config_excel/equipment.xlsx
+++ b/space-battleship/config_excel/equipment.xlsx
@@ -1380,7 +1380,7 @@
         <v>0.2</v>
       </c>
       <c r="G6" s="0" t="n">
-        <v>1.5</v>
+        <v>1.4</v>
       </c>
       <c r="I6" s="0" t="n">
         <v>1</v>
@@ -1413,7 +1413,7 @@
         <v>2</v>
       </c>
       <c r="E7" s="0" t="n">
-        <v>160</v>
+        <v>200</v>
       </c>
       <c r="F7" s="0" t="n">
         <v>0.2</v>
@@ -1431,7 +1431,7 @@
         <v>0.2</v>
       </c>
       <c r="O7" s="0" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="P7" s="0" t="n">
         <v>30</v>

</xml_diff>

<commit_message>
Restore fixed weapon baseline and park unapproved candidates
</commit_message>
<xml_diff>
--- a/space-battleship/config_excel/equipment.xlsx
+++ b/space-battleship/config_excel/equipment.xlsx
@@ -1380,7 +1380,7 @@
         <v>0.2</v>
       </c>
       <c r="G6" s="0" t="n">
-        <v>1.4</v>
+        <v>1.5</v>
       </c>
       <c r="I6" s="0" t="n">
         <v>1</v>
@@ -1431,7 +1431,7 @@
         <v>0.2</v>
       </c>
       <c r="O7" s="0" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="P7" s="0" t="n">
         <v>30</v>

</xml_diff>

<commit_message>
Mount opening growth candidate with frozen reward references
</commit_message>
<xml_diff>
--- a/space-battleship/config_excel/equipment.xlsx
+++ b/space-battleship/config_excel/equipment.xlsx
@@ -1373,8 +1373,8 @@
       <c r="D6" s="0" t="n">
         <v>1</v>
       </c>
-      <c r="E6" s="0" t="n">
-        <v>300</v>
+      <c r="E6" s="0">
+        <v>350</v>
       </c>
       <c r="F6" s="0" t="n">
         <v>0.2</v>
@@ -1412,8 +1412,8 @@
       <c r="D7" s="0" t="n">
         <v>2</v>
       </c>
-      <c r="E7" s="0" t="n">
-        <v>200</v>
+      <c r="E7" s="0">
+        <v>170</v>
       </c>
       <c r="F7" s="0" t="n">
         <v>0.2</v>
@@ -1454,8 +1454,8 @@
       <c r="D8" s="0" t="n">
         <v>2</v>
       </c>
-      <c r="E8" s="0" t="n">
-        <v>1500</v>
+      <c r="E8" s="0">
+        <v>1200</v>
       </c>
       <c r="F8" s="0" t="n">
         <v>0.2</v>
@@ -1583,8 +1583,8 @@
       <c r="F12" s="0" t="n">
         <v>0.2</v>
       </c>
-      <c r="G12" s="0" t="n">
-        <v>0.28</v>
+      <c r="G12" s="0">
+        <v>0.25</v>
       </c>
       <c r="I12" s="0" t="n">
         <v>1</v>

</xml_diff>

<commit_message>
fix: restore visible pulse projectile speed
</commit_message>
<xml_diff>
--- a/space-battleship/config_excel/equipment.xlsx
+++ b/space-battleship/config_excel/equipment.xlsx
@@ -1373,7 +1373,7 @@
       <c r="D6" s="0" t="n">
         <v>1</v>
       </c>
-      <c r="E6" s="0">
+      <c r="E6" s="0" t="n">
         <v>350</v>
       </c>
       <c r="F6" s="0" t="n">
@@ -1392,7 +1392,7 @@
         <v>0.2</v>
       </c>
       <c r="O6" s="0" t="n">
-        <v>10000</v>
+        <v>30</v>
       </c>
     </row>
     <row r="7">
@@ -1412,7 +1412,7 @@
       <c r="D7" s="0" t="n">
         <v>2</v>
       </c>
-      <c r="E7" s="0">
+      <c r="E7" s="0" t="n">
         <v>170</v>
       </c>
       <c r="F7" s="0" t="n">
@@ -1454,7 +1454,7 @@
       <c r="D8" s="0" t="n">
         <v>2</v>
       </c>
-      <c r="E8" s="0">
+      <c r="E8" s="0" t="n">
         <v>1200</v>
       </c>
       <c r="F8" s="0" t="n">
@@ -1583,7 +1583,7 @@
       <c r="F12" s="0" t="n">
         <v>0.2</v>
       </c>
-      <c r="G12" s="0">
+      <c r="G12" s="0" t="n">
         <v>0.25</v>
       </c>
       <c r="I12" s="0" t="n">

</xml_diff>

<commit_message>
Set player shield to 75% armor capacity and revise early growth plan
</commit_message>
<xml_diff>
--- a/space-battleship/config_excel/equipment.xlsx
+++ b/space-battleship/config_excel/equipment.xlsx
@@ -1319,7 +1319,7 @@
       </c>
       <c r="B5" s="0" t="inlineStr">
         <is>
-          <t>这个是飞船的基础护盾，护盾会先于护甲被扣除，同时护盾会缓慢恢复。额外参数para1是护盾值，para2是每秒恢复的比例，para3是连续多少秒不受攻击后才开始恢复，被攻击会立即停止恢复，dmgtype表明护盾对这个类型的伤害有减伤,para4是para1随等级的增加值,算法为para1*(1+para4)^(等级-1),除了首2位其他位都是0,四舍五入,如果不足100,则末尾为5</t>
+          <t>飞船基础护盾，先于装甲承伤；dmgtype为其抗性类型。para1是1级容量；同等级容量取装甲按原规则取整后的数值，再乘para1/装甲para1，确保所有等级维持同一比例。para2为每秒恢复最大容量的比例，para3为每次受击后等待秒数；para4须与装甲成长率一致，供导入校验。</t>
         </is>
       </c>
       <c r="C5" s="0" t="n">
@@ -1344,7 +1344,7 @@
         <v>0.2</v>
       </c>
       <c r="O5" s="0" t="n">
-        <v>500</v>
+        <v>750</v>
       </c>
       <c r="P5" s="0" t="n">
         <v>0.3</v>

</xml_diff>

<commit_message>
Implement approved first-three-stage growth and enemy pacing
</commit_message>
<xml_diff>
--- a/space-battleship/config_excel/equipment.xlsx
+++ b/space-battleship/config_excel/equipment.xlsx
@@ -1001,7 +1001,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R13"/>
+  <dimension ref="A1:R14"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="14.4"/>
   <cols>
     <col width="13" customWidth="1" style="1" min="1" max="1"/>
@@ -1650,6 +1650,33 @@
         <v>1</v>
       </c>
     </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>laser-mon</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>敌方低频单发能量激光；para1 为飞行速度，冷却用于留出玩家护盾恢复窗口。</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>1</v>
+      </c>
+      <c r="D14" t="n">
+        <v>1</v>
+      </c>
+      <c r="E14" t="n">
+        <v>80</v>
+      </c>
+      <c r="G14" t="n">
+        <v>3.6</v>
+      </c>
+      <c r="O14" t="n">
+        <v>20</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" paperSize="9"/>

</xml_diff>